<commit_message>
Update README and evaluation results
</commit_message>
<xml_diff>
--- a/evaluation/hasil_evaluasi.xlsx
+++ b/evaluation/hasil_evaluasi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghofu\RAG-UTS-Kelompok 5\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E5D8C92-63C6-4867-9AE0-B186BEED3AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F522CD36-1F46-4E69-BC72-F3E8E84850BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{08DBF7F2-BF50-4D31-9DCF-A6782C52167D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{08DBF7F2-BF50-4D31-9DCF-A6782C52167D}"/>
   </bookViews>
   <sheets>
     <sheet name="Lembar1" sheetId="1" r:id="rId1"/>

</xml_diff>